<commit_message>
DP: create_forecast_basic - utils - monitoring_df.ipynb - pop division total_emp in 2020
</commit_message>
<xml_diff>
--- a/create_forecast_basic/utils/monitoring_df_fixed_6.xlsx
+++ b/create_forecast_basic/utils/monitoring_df_fixed_6.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1529" uniqueCount="1509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1536" uniqueCount="1516">
   <si>
     <t>2020</t>
   </si>
@@ -3166,31 +3166,31 @@
     <t>emp_okev at הר אדר in 2050</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>emp_okev at הר חברון_x000D_
+    <t>emp_okev at הר חברון_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3236,31 +3236,31 @@
     <t>emp_okev at מבשרת ציון in 2050</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>emp_okev at מגילות ים המלח_x000D_
+    <t>emp_okev at מגילות ים המלח_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3411,31 +3411,31 @@
     <t>emp_okev at עמנואל in 2050</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>emp_okev at ערבות הירדן_x000D_
+    <t>emp_okev at ערבות הירדן_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3817,31 +3817,31 @@
     <t>total_emp at הר אדר in 2050</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>total_emp at הר חברון_x000D_
+    <t>total_emp at הר חברון_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -3887,31 +3887,31 @@
     <t>total_emp at מבשרת ציון in 2050</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>total_emp at מגילות ים המלח_x000D_
+    <t>total_emp at מגילות ים המלח_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -4062,31 +4062,31 @@
     <t>total_emp at עמנואל in 2050</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2020</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2025</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2030</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2035</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2040</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2045</t>
   </si>
   <si>
-    <t>total_emp at ערבות הירדן_x000D_
+    <t>total_emp at ערבות הירדן_x005F_x000D_
  in 2050</t>
   </si>
   <si>
@@ -4529,6 +4529,27 @@
   </si>
   <si>
     <t>pop division emp_okev at תלפיות מזרח in 2025</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2020</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2025</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2030</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2035</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2040</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2045</t>
+  </si>
+  <si>
+    <t>pop division total_emp in 2050</t>
   </si>
   <si>
     <t>1,758,461</t>
@@ -4940,7 +4961,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1488"/>
+  <dimension ref="A1:E1495"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4962,16 +4983,16 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>1491</v>
+        <v>1498</v>
       </c>
       <c r="C2" t="s">
-        <v>1491</v>
+        <v>1498</v>
       </c>
       <c r="D2" t="s">
-        <v>1491</v>
+        <v>1498</v>
       </c>
       <c r="E2" t="s">
-        <v>1491</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -4979,13 +5000,13 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>1496</v>
+        <v>1503</v>
       </c>
       <c r="D3" t="s">
-        <v>1501</v>
+        <v>1508</v>
       </c>
       <c r="E3" t="s">
-        <v>1505</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -4993,16 +5014,16 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>1492</v>
+        <v>1499</v>
       </c>
       <c r="C4" t="s">
-        <v>1492</v>
+        <v>1499</v>
       </c>
       <c r="D4" t="s">
-        <v>1492</v>
+        <v>1499</v>
       </c>
       <c r="E4" t="s">
-        <v>1492</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -5010,13 +5031,13 @@
         <v>7</v>
       </c>
       <c r="C5" t="s">
-        <v>1497</v>
+        <v>1504</v>
       </c>
       <c r="D5" t="s">
-        <v>1502</v>
+        <v>1509</v>
       </c>
       <c r="E5" t="s">
-        <v>1506</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -5109,16 +5130,16 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
       <c r="C11" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
       <c r="D11" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
       <c r="E11" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -5126,13 +5147,13 @@
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
       <c r="D12" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
       <c r="E12" t="s">
-        <v>1493</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -5140,16 +5161,16 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>1494</v>
+        <v>1501</v>
       </c>
       <c r="C13" t="s">
-        <v>1494</v>
+        <v>1501</v>
       </c>
       <c r="D13" t="s">
-        <v>1494</v>
+        <v>1501</v>
       </c>
       <c r="E13" t="s">
-        <v>1494</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -5157,13 +5178,13 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>1498</v>
+        <v>1505</v>
       </c>
       <c r="D14" t="s">
-        <v>1503</v>
+        <v>1510</v>
       </c>
       <c r="E14" t="s">
-        <v>1507</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -5171,16 +5192,16 @@
         <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>1495</v>
+        <v>1502</v>
       </c>
       <c r="C15" t="s">
-        <v>1495</v>
+        <v>1502</v>
       </c>
       <c r="D15" t="s">
-        <v>1495</v>
+        <v>1502</v>
       </c>
       <c r="E15" t="s">
-        <v>1495</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -5188,13 +5209,13 @@
         <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>1499</v>
+        <v>1506</v>
       </c>
       <c r="D16" t="s">
-        <v>1504</v>
+        <v>1511</v>
       </c>
       <c r="E16" t="s">
-        <v>1508</v>
+        <v>1515</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -5355,10 +5376,10 @@
         <v>28</v>
       </c>
       <c r="C26">
-        <v>188.1410644079084</v>
+        <v>188.1410644079083</v>
       </c>
       <c r="D26">
-        <v>183.9696620191286</v>
+        <v>183.9696620191285</v>
       </c>
       <c r="E26">
         <v>185.6774324006336</v>
@@ -5635,13 +5656,13 @@
         <v>48</v>
       </c>
       <c r="C46" t="s">
-        <v>1500</v>
+        <v>1507</v>
       </c>
       <c r="D46" t="s">
-        <v>1500</v>
+        <v>1507</v>
       </c>
       <c r="E46" t="s">
-        <v>1500</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -25830,6 +25851,104 @@
       </c>
       <c r="E1488">
         <v>5.208887551814326</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:5">
+      <c r="A1489" s="1" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C1489">
+        <v>0.274510590027404</v>
+      </c>
+      <c r="D1489">
+        <v>0.274510590027404</v>
+      </c>
+      <c r="E1489">
+        <v>0.274510590027404</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:5">
+      <c r="A1490" s="1" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C1490">
+        <v>0.1085610779961064</v>
+      </c>
+      <c r="D1490">
+        <v>0.1042627101407602</v>
+      </c>
+      <c r="E1490">
+        <v>0.1051127003854925</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:5">
+      <c r="A1491" s="1" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C1491">
+        <v>0.1125054369322683</v>
+      </c>
+      <c r="D1491">
+        <v>0.1060000485240958</v>
+      </c>
+      <c r="E1491">
+        <v>0.108259127712942</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:5">
+      <c r="A1492" s="1" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C1492">
+        <v>0.117776582480796</v>
+      </c>
+      <c r="D1492">
+        <v>0.1088794149716449</v>
+      </c>
+      <c r="E1492">
+        <v>0.1124915624920027</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:5">
+      <c r="A1493" s="1" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C1493">
+        <v>0.1227534623323177</v>
+      </c>
+      <c r="D1493">
+        <v>0.1111431609688907</v>
+      </c>
+      <c r="E1493">
+        <v>0.1165598777550276</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:5">
+      <c r="A1494" s="1" t="s">
+        <v>1496</v>
+      </c>
+      <c r="C1494">
+        <v>0.1292444792424143</v>
+      </c>
+      <c r="D1494">
+        <v>0.1129801244081925</v>
+      </c>
+      <c r="E1494">
+        <v>0.1202497001616002</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:5">
+      <c r="A1495" s="1" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C1495">
+        <v>0.1309869731098417</v>
+      </c>
+      <c r="D1495">
+        <v>0.1150036371136272</v>
+      </c>
+      <c r="E1495">
+        <v>0.1240135292494374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>